<commit_message>
Reset Excel Table for CNC3X-05
</commit_message>
<xml_diff>
--- a/FM-MN-07_CNC3X-05.xlsx
+++ b/FM-MN-07_CNC3X-05.xlsx
@@ -1804,11 +1804,7 @@
           <t>Worm up เครื่องจักร 15 นาที ทุกครั้งที่ใช้งาน</t>
         </is>
       </c>
-      <c r="C6" s="23" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="C6" s="23" t="inlineStr"/>
       <c r="D6" s="22" t="inlineStr"/>
       <c r="E6" s="22" t="inlineStr"/>
       <c r="F6" s="22" t="inlineStr"/>
@@ -1849,11 +1845,7 @@
           <t>เช็คระดับนำมันที่ Pump Hydraulic ทุกวัน เติมเมื่อพร่อง</t>
         </is>
       </c>
-      <c r="C7" s="23" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="C7" s="23" t="inlineStr"/>
       <c r="D7" s="22" t="inlineStr"/>
       <c r="E7" s="22" t="inlineStr"/>
       <c r="F7" s="22" t="inlineStr"/>
@@ -1935,11 +1927,7 @@
           <t>ตรวจเช็คแรงดัน Air Control Unit ปกติเฉลี่ยที่ 0.5 Mpa</t>
         </is>
       </c>
-      <c r="C9" s="23" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="C9" s="23" t="inlineStr"/>
       <c r="D9" s="22" t="inlineStr"/>
       <c r="E9" s="22" t="inlineStr"/>
       <c r="F9" s="22" t="inlineStr"/>
@@ -2021,11 +2009,7 @@
           <t>อัดจารบี Ballscrew และ Linear Guideทุก 1ครั้งต่อเดือน</t>
         </is>
       </c>
-      <c r="C11" s="23" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+      <c r="C11" s="23" t="inlineStr"/>
       <c r="D11" s="22" t="inlineStr"/>
       <c r="E11" s="22" t="inlineStr"/>
       <c r="F11" s="22" t="inlineStr"/>
@@ -2148,11 +2132,7 @@
           <t>การทำงานของ Coolant pump</t>
         </is>
       </c>
-      <c r="C14" s="23" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="C14" s="23" t="inlineStr"/>
       <c r="D14" s="22" t="inlineStr"/>
       <c r="E14" s="22" t="inlineStr"/>
       <c r="F14" s="22" t="inlineStr"/>
@@ -2193,11 +2173,7 @@
           <t>การทำงานของ Unclamp และการเปลี่ยน Tool</t>
         </is>
       </c>
-      <c r="C15" s="23" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="C15" s="23" t="inlineStr"/>
       <c r="D15" s="22" t="inlineStr"/>
       <c r="E15" s="22" t="inlineStr"/>
       <c r="F15" s="22" t="inlineStr"/>
@@ -2238,11 +2214,7 @@
           <t>การทำงานของ Spindle</t>
         </is>
       </c>
-      <c r="C16" s="23" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="C16" s="23" t="inlineStr"/>
       <c r="D16" s="22" t="inlineStr"/>
       <c r="E16" s="22" t="inlineStr"/>
       <c r="F16" s="22" t="inlineStr"/>
@@ -2283,11 +2255,7 @@
           <t>การทำงานของ Arm เปลี่ยน Tool</t>
         </is>
       </c>
-      <c r="C17" s="23" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="C17" s="23" t="inlineStr"/>
       <c r="D17" s="22" t="inlineStr"/>
       <c r="E17" s="22" t="inlineStr"/>
       <c r="F17" s="22" t="inlineStr"/>
@@ -2328,11 +2296,7 @@
           <t>ตรวจสอบระดับของน้ำ Coolant เติมเมื่ออยู่ระดับที่ต่ำ</t>
         </is>
       </c>
-      <c r="C18" s="23" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="C18" s="23" t="inlineStr"/>
       <c r="D18" s="22" t="inlineStr"/>
       <c r="E18" s="22" t="inlineStr"/>
       <c r="F18" s="22" t="inlineStr"/>
@@ -2373,11 +2337,7 @@
           <t>ความสะอาดทั่วไปของเครื่องจักรโดยรวม</t>
         </is>
       </c>
-      <c r="C19" s="23" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="C19" s="23" t="inlineStr"/>
       <c r="D19" s="22" t="inlineStr"/>
       <c r="E19" s="22" t="inlineStr"/>
       <c r="F19" s="22" t="inlineStr"/>
@@ -2418,11 +2378,7 @@
           <t>ตรวจสอบความพร้อมสภาพโดยรวม(ฟังด้วยหู ดูด้วยตา)</t>
         </is>
       </c>
-      <c r="C20" s="23" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="C20" s="23" t="inlineStr"/>
       <c r="D20" s="22" t="inlineStr"/>
       <c r="E20" s="22" t="inlineStr"/>
       <c r="F20" s="22" t="inlineStr"/>
@@ -2463,11 +2419,7 @@
           <t>ตรวจสอบสายไฮโดรลิกส์ และสายลม</t>
         </is>
       </c>
-      <c r="C21" s="23" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="C21" s="23" t="inlineStr"/>
       <c r="D21" s="22" t="inlineStr"/>
       <c r="E21" s="22" t="inlineStr"/>
       <c r="F21" s="22" t="inlineStr"/>
@@ -2502,11 +2454,7 @@
     <row r="22" ht="22.5" customHeight="1">
       <c r="A22" s="3" t="n"/>
       <c r="B22" s="8" t="n"/>
-      <c r="C22" s="33" t="inlineStr">
-        <is>
-          <t>นาย ทินภัทร สียางนอก</t>
-        </is>
-      </c>
+      <c r="C22" s="33" t="inlineStr"/>
       <c r="D22" s="28" t="inlineStr"/>
       <c r="E22" s="28" t="inlineStr"/>
       <c r="F22" s="28" t="inlineStr"/>

</xml_diff>

<commit_message>
Direct Write Excel for CNC3X-05 Day 6
</commit_message>
<xml_diff>
--- a/FM-MN-07_CNC3X-05.xlsx
+++ b/FM-MN-07_CNC3X-05.xlsx
@@ -1809,7 +1809,11 @@
       <c r="E6" s="22" t="inlineStr"/>
       <c r="F6" s="22" t="inlineStr"/>
       <c r="G6" s="22" t="inlineStr"/>
-      <c r="H6" s="22" t="inlineStr"/>
+      <c r="H6" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I6" s="22" t="inlineStr"/>
       <c r="J6" s="22" t="inlineStr"/>
       <c r="K6" s="22" t="inlineStr"/>
@@ -1850,7 +1854,11 @@
       <c r="E7" s="22" t="inlineStr"/>
       <c r="F7" s="22" t="inlineStr"/>
       <c r="G7" s="22" t="inlineStr"/>
-      <c r="H7" s="22" t="inlineStr"/>
+      <c r="H7" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I7" s="22" t="inlineStr"/>
       <c r="J7" s="22" t="inlineStr"/>
       <c r="K7" s="22" t="inlineStr"/>
@@ -1891,7 +1899,11 @@
       <c r="E8" s="22" t="inlineStr"/>
       <c r="F8" s="22" t="inlineStr"/>
       <c r="G8" s="22" t="inlineStr"/>
-      <c r="H8" s="22" t="inlineStr"/>
+      <c r="H8" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I8" s="22" t="inlineStr"/>
       <c r="J8" s="22" t="inlineStr"/>
       <c r="K8" s="22" t="inlineStr"/>
@@ -1932,7 +1944,11 @@
       <c r="E9" s="22" t="inlineStr"/>
       <c r="F9" s="22" t="inlineStr"/>
       <c r="G9" s="22" t="inlineStr"/>
-      <c r="H9" s="22" t="inlineStr"/>
+      <c r="H9" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I9" s="22" t="inlineStr"/>
       <c r="J9" s="22" t="inlineStr"/>
       <c r="K9" s="22" t="inlineStr"/>
@@ -1973,7 +1989,11 @@
       <c r="E10" s="22" t="inlineStr"/>
       <c r="F10" s="22" t="inlineStr"/>
       <c r="G10" s="22" t="inlineStr"/>
-      <c r="H10" s="22" t="inlineStr"/>
+      <c r="H10" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I10" s="22" t="inlineStr"/>
       <c r="J10" s="22" t="inlineStr"/>
       <c r="K10" s="22" t="inlineStr"/>
@@ -2014,7 +2034,11 @@
       <c r="E11" s="22" t="inlineStr"/>
       <c r="F11" s="22" t="inlineStr"/>
       <c r="G11" s="22" t="inlineStr"/>
-      <c r="H11" s="22" t="inlineStr"/>
+      <c r="H11" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I11" s="22" t="inlineStr"/>
       <c r="J11" s="22" t="inlineStr"/>
       <c r="K11" s="22" t="inlineStr"/>
@@ -2055,7 +2079,11 @@
       <c r="E12" s="22" t="inlineStr"/>
       <c r="F12" s="22" t="inlineStr"/>
       <c r="G12" s="22" t="inlineStr"/>
-      <c r="H12" s="22" t="inlineStr"/>
+      <c r="H12" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I12" s="22" t="inlineStr"/>
       <c r="J12" s="22" t="inlineStr"/>
       <c r="K12" s="22" t="inlineStr"/>
@@ -2096,7 +2124,11 @@
       <c r="E13" s="22" t="inlineStr"/>
       <c r="F13" s="22" t="inlineStr"/>
       <c r="G13" s="22" t="inlineStr"/>
-      <c r="H13" s="22" t="inlineStr"/>
+      <c r="H13" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I13" s="22" t="inlineStr"/>
       <c r="J13" s="22" t="inlineStr"/>
       <c r="K13" s="22" t="inlineStr"/>
@@ -2137,7 +2169,11 @@
       <c r="E14" s="22" t="inlineStr"/>
       <c r="F14" s="22" t="inlineStr"/>
       <c r="G14" s="22" t="inlineStr"/>
-      <c r="H14" s="22" t="inlineStr"/>
+      <c r="H14" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I14" s="22" t="inlineStr"/>
       <c r="J14" s="22" t="inlineStr"/>
       <c r="K14" s="22" t="inlineStr"/>
@@ -2178,7 +2214,11 @@
       <c r="E15" s="22" t="inlineStr"/>
       <c r="F15" s="22" t="inlineStr"/>
       <c r="G15" s="22" t="inlineStr"/>
-      <c r="H15" s="22" t="inlineStr"/>
+      <c r="H15" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I15" s="22" t="inlineStr"/>
       <c r="J15" s="22" t="inlineStr"/>
       <c r="K15" s="22" t="inlineStr"/>
@@ -2219,7 +2259,11 @@
       <c r="E16" s="22" t="inlineStr"/>
       <c r="F16" s="22" t="inlineStr"/>
       <c r="G16" s="22" t="inlineStr"/>
-      <c r="H16" s="22" t="inlineStr"/>
+      <c r="H16" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I16" s="22" t="inlineStr"/>
       <c r="J16" s="22" t="inlineStr"/>
       <c r="K16" s="22" t="inlineStr"/>
@@ -2260,7 +2304,11 @@
       <c r="E17" s="22" t="inlineStr"/>
       <c r="F17" s="22" t="inlineStr"/>
       <c r="G17" s="22" t="inlineStr"/>
-      <c r="H17" s="22" t="inlineStr"/>
+      <c r="H17" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I17" s="22" t="inlineStr"/>
       <c r="J17" s="22" t="inlineStr"/>
       <c r="K17" s="22" t="inlineStr"/>
@@ -2301,7 +2349,11 @@
       <c r="E18" s="22" t="inlineStr"/>
       <c r="F18" s="22" t="inlineStr"/>
       <c r="G18" s="22" t="inlineStr"/>
-      <c r="H18" s="22" t="inlineStr"/>
+      <c r="H18" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I18" s="22" t="inlineStr"/>
       <c r="J18" s="22" t="inlineStr"/>
       <c r="K18" s="22" t="inlineStr"/>
@@ -2342,7 +2394,11 @@
       <c r="E19" s="22" t="inlineStr"/>
       <c r="F19" s="22" t="inlineStr"/>
       <c r="G19" s="22" t="inlineStr"/>
-      <c r="H19" s="22" t="inlineStr"/>
+      <c r="H19" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I19" s="22" t="inlineStr"/>
       <c r="J19" s="22" t="inlineStr"/>
       <c r="K19" s="22" t="inlineStr"/>
@@ -2383,7 +2439,11 @@
       <c r="E20" s="22" t="inlineStr"/>
       <c r="F20" s="22" t="inlineStr"/>
       <c r="G20" s="22" t="inlineStr"/>
-      <c r="H20" s="22" t="inlineStr"/>
+      <c r="H20" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I20" s="22" t="inlineStr"/>
       <c r="J20" s="22" t="inlineStr"/>
       <c r="K20" s="22" t="inlineStr"/>
@@ -2424,7 +2484,11 @@
       <c r="E21" s="22" t="inlineStr"/>
       <c r="F21" s="22" t="inlineStr"/>
       <c r="G21" s="22" t="inlineStr"/>
-      <c r="H21" s="22" t="inlineStr"/>
+      <c r="H21" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I21" s="22" t="inlineStr"/>
       <c r="J21" s="22" t="inlineStr"/>
       <c r="K21" s="22" t="inlineStr"/>
@@ -2459,7 +2523,11 @@
       <c r="E22" s="28" t="inlineStr"/>
       <c r="F22" s="28" t="inlineStr"/>
       <c r="G22" s="28" t="inlineStr"/>
-      <c r="H22" s="28" t="inlineStr"/>
+      <c r="H22" s="33" t="inlineStr">
+        <is>
+          <t>ณัช วกรัยเจริญ</t>
+        </is>
+      </c>
       <c r="I22" s="28" t="inlineStr"/>
       <c r="J22" s="28" t="inlineStr"/>
       <c r="K22" s="28" t="inlineStr"/>

</xml_diff>

<commit_message>
Safe Direct Write Excel for CNC3X-05 Day 7
</commit_message>
<xml_diff>
--- a/FM-MN-07_CNC3X-05.xlsx
+++ b/FM-MN-07_CNC3X-05.xlsx
@@ -1814,7 +1814,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I6" s="22" t="inlineStr"/>
+      <c r="I6" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J6" s="22" t="inlineStr"/>
       <c r="K6" s="22" t="inlineStr"/>
       <c r="L6" s="22" t="inlineStr"/>
@@ -1859,7 +1863,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I7" s="22" t="inlineStr"/>
+      <c r="I7" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J7" s="22" t="inlineStr"/>
       <c r="K7" s="22" t="inlineStr"/>
       <c r="L7" s="22" t="inlineStr"/>
@@ -1904,7 +1912,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I8" s="22" t="inlineStr"/>
+      <c r="I8" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J8" s="22" t="inlineStr"/>
       <c r="K8" s="22" t="inlineStr"/>
       <c r="L8" s="22" t="inlineStr"/>
@@ -1949,7 +1961,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I9" s="22" t="inlineStr"/>
+      <c r="I9" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J9" s="22" t="inlineStr"/>
       <c r="K9" s="22" t="inlineStr"/>
       <c r="L9" s="22" t="inlineStr"/>
@@ -1994,7 +2010,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I10" s="22" t="inlineStr"/>
+      <c r="I10" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J10" s="22" t="inlineStr"/>
       <c r="K10" s="22" t="inlineStr"/>
       <c r="L10" s="22" t="inlineStr"/>
@@ -2039,7 +2059,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I11" s="22" t="inlineStr"/>
+      <c r="I11" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J11" s="22" t="inlineStr"/>
       <c r="K11" s="22" t="inlineStr"/>
       <c r="L11" s="22" t="inlineStr"/>
@@ -2084,7 +2108,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I12" s="22" t="inlineStr"/>
+      <c r="I12" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J12" s="22" t="inlineStr"/>
       <c r="K12" s="22" t="inlineStr"/>
       <c r="L12" s="22" t="inlineStr"/>
@@ -2129,7 +2157,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I13" s="22" t="inlineStr"/>
+      <c r="I13" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J13" s="22" t="inlineStr"/>
       <c r="K13" s="22" t="inlineStr"/>
       <c r="L13" s="22" t="inlineStr"/>
@@ -2174,7 +2206,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I14" s="22" t="inlineStr"/>
+      <c r="I14" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J14" s="22" t="inlineStr"/>
       <c r="K14" s="22" t="inlineStr"/>
       <c r="L14" s="22" t="inlineStr"/>
@@ -2219,7 +2255,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I15" s="22" t="inlineStr"/>
+      <c r="I15" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J15" s="22" t="inlineStr"/>
       <c r="K15" s="22" t="inlineStr"/>
       <c r="L15" s="22" t="inlineStr"/>
@@ -2264,7 +2304,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I16" s="22" t="inlineStr"/>
+      <c r="I16" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J16" s="22" t="inlineStr"/>
       <c r="K16" s="22" t="inlineStr"/>
       <c r="L16" s="22" t="inlineStr"/>
@@ -2309,7 +2353,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I17" s="22" t="inlineStr"/>
+      <c r="I17" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J17" s="22" t="inlineStr"/>
       <c r="K17" s="22" t="inlineStr"/>
       <c r="L17" s="22" t="inlineStr"/>
@@ -2354,7 +2402,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I18" s="22" t="inlineStr"/>
+      <c r="I18" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J18" s="22" t="inlineStr"/>
       <c r="K18" s="22" t="inlineStr"/>
       <c r="L18" s="22" t="inlineStr"/>
@@ -2399,7 +2451,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I19" s="22" t="inlineStr"/>
+      <c r="I19" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J19" s="22" t="inlineStr"/>
       <c r="K19" s="22" t="inlineStr"/>
       <c r="L19" s="22" t="inlineStr"/>
@@ -2444,7 +2500,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I20" s="22" t="inlineStr"/>
+      <c r="I20" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J20" s="22" t="inlineStr"/>
       <c r="K20" s="22" t="inlineStr"/>
       <c r="L20" s="22" t="inlineStr"/>
@@ -2489,7 +2549,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I21" s="22" t="inlineStr"/>
+      <c r="I21" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J21" s="22" t="inlineStr"/>
       <c r="K21" s="22" t="inlineStr"/>
       <c r="L21" s="22" t="inlineStr"/>
@@ -2528,7 +2592,11 @@
           <t>ณัช วกรัยเจริญ</t>
         </is>
       </c>
-      <c r="I22" s="28" t="inlineStr"/>
+      <c r="I22" s="33" t="inlineStr">
+        <is>
+          <t>ณัช วิกรัยเจริญ</t>
+        </is>
+      </c>
       <c r="J22" s="28" t="inlineStr"/>
       <c r="K22" s="28" t="inlineStr"/>
       <c r="L22" s="28" t="inlineStr"/>
@@ -2667,7 +2735,11 @@
       <c r="Y27" s="21" t="n"/>
     </row>
     <row r="28" ht="173.25" customHeight="1">
-      <c r="B28" s="46" t="inlineStr"/>
+      <c r="B28" s="46" t="inlineStr">
+        <is>
+          <t>[วันที่ 7]: ข้อ 7: แกนzมีเสียงดัง</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="21" customHeight="1">
       <c r="AA29" s="19" t="n"/>

</xml_diff>

<commit_message>
Safe Direct Write Excel for CNC3X-05 Day 8
</commit_message>
<xml_diff>
--- a/FM-MN-07_CNC3X-05.xlsx
+++ b/FM-MN-07_CNC3X-05.xlsx
@@ -1819,7 +1819,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J6" s="22" t="inlineStr"/>
+      <c r="J6" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K6" s="22" t="inlineStr"/>
       <c r="L6" s="22" t="inlineStr"/>
       <c r="M6" s="22" t="inlineStr"/>
@@ -1868,7 +1872,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J7" s="22" t="inlineStr"/>
+      <c r="J7" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K7" s="22" t="inlineStr"/>
       <c r="L7" s="22" t="inlineStr"/>
       <c r="M7" s="22" t="inlineStr"/>
@@ -1917,7 +1925,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J8" s="22" t="inlineStr"/>
+      <c r="J8" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K8" s="22" t="inlineStr"/>
       <c r="L8" s="22" t="inlineStr"/>
       <c r="M8" s="22" t="inlineStr"/>
@@ -1966,7 +1978,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J9" s="22" t="inlineStr"/>
+      <c r="J9" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K9" s="22" t="inlineStr"/>
       <c r="L9" s="22" t="inlineStr"/>
       <c r="M9" s="22" t="inlineStr"/>
@@ -2015,7 +2031,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J10" s="22" t="inlineStr"/>
+      <c r="J10" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K10" s="22" t="inlineStr"/>
       <c r="L10" s="22" t="inlineStr"/>
       <c r="M10" s="22" t="inlineStr"/>
@@ -2064,7 +2084,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J11" s="22" t="inlineStr"/>
+      <c r="J11" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K11" s="22" t="inlineStr"/>
       <c r="L11" s="22" t="inlineStr"/>
       <c r="M11" s="22" t="inlineStr"/>
@@ -2113,7 +2137,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J12" s="22" t="inlineStr"/>
+      <c r="J12" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K12" s="22" t="inlineStr"/>
       <c r="L12" s="22" t="inlineStr"/>
       <c r="M12" s="22" t="inlineStr"/>
@@ -2162,7 +2190,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J13" s="22" t="inlineStr"/>
+      <c r="J13" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K13" s="22" t="inlineStr"/>
       <c r="L13" s="22" t="inlineStr"/>
       <c r="M13" s="22" t="inlineStr"/>
@@ -2211,7 +2243,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J14" s="22" t="inlineStr"/>
+      <c r="J14" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K14" s="22" t="inlineStr"/>
       <c r="L14" s="22" t="inlineStr"/>
       <c r="M14" s="22" t="inlineStr"/>
@@ -2260,7 +2296,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J15" s="22" t="inlineStr"/>
+      <c r="J15" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K15" s="22" t="inlineStr"/>
       <c r="L15" s="22" t="inlineStr"/>
       <c r="M15" s="22" t="inlineStr"/>
@@ -2309,7 +2349,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J16" s="22" t="inlineStr"/>
+      <c r="J16" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K16" s="22" t="inlineStr"/>
       <c r="L16" s="22" t="inlineStr"/>
       <c r="M16" s="22" t="inlineStr"/>
@@ -2358,7 +2402,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J17" s="22" t="inlineStr"/>
+      <c r="J17" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K17" s="22" t="inlineStr"/>
       <c r="L17" s="22" t="inlineStr"/>
       <c r="M17" s="22" t="inlineStr"/>
@@ -2407,7 +2455,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J18" s="22" t="inlineStr"/>
+      <c r="J18" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K18" s="22" t="inlineStr"/>
       <c r="L18" s="22" t="inlineStr"/>
       <c r="M18" s="22" t="inlineStr"/>
@@ -2456,7 +2508,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J19" s="22" t="inlineStr"/>
+      <c r="J19" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K19" s="22" t="inlineStr"/>
       <c r="L19" s="22" t="inlineStr"/>
       <c r="M19" s="22" t="inlineStr"/>
@@ -2505,7 +2561,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J20" s="22" t="inlineStr"/>
+      <c r="J20" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K20" s="22" t="inlineStr"/>
       <c r="L20" s="22" t="inlineStr"/>
       <c r="M20" s="22" t="inlineStr"/>
@@ -2554,7 +2614,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J21" s="22" t="inlineStr"/>
+      <c r="J21" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K21" s="22" t="inlineStr"/>
       <c r="L21" s="22" t="inlineStr"/>
       <c r="M21" s="22" t="inlineStr"/>
@@ -2597,7 +2661,11 @@
           <t>ณัช วิกรัยเจริญ</t>
         </is>
       </c>
-      <c r="J22" s="28" t="inlineStr"/>
+      <c r="J22" s="33" t="inlineStr">
+        <is>
+          <t>ณัช วิกรัยเจริญ</t>
+        </is>
+      </c>
       <c r="K22" s="28" t="inlineStr"/>
       <c r="L22" s="28" t="inlineStr"/>
       <c r="M22" s="28" t="inlineStr"/>

</xml_diff>

<commit_message>
Safe Direct Write Excel for CNC3X-05 Day 10
</commit_message>
<xml_diff>
--- a/FM-MN-07_CNC3X-05.xlsx
+++ b/FM-MN-07_CNC3X-05.xlsx
@@ -1825,7 +1825,11 @@
         </is>
       </c>
       <c r="K6" s="22" t="inlineStr"/>
-      <c r="L6" s="22" t="inlineStr"/>
+      <c r="L6" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M6" s="22" t="inlineStr"/>
       <c r="N6" s="22" t="inlineStr"/>
       <c r="O6" s="22" t="inlineStr"/>
@@ -1878,7 +1882,11 @@
         </is>
       </c>
       <c r="K7" s="22" t="inlineStr"/>
-      <c r="L7" s="22" t="inlineStr"/>
+      <c r="L7" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M7" s="22" t="inlineStr"/>
       <c r="N7" s="22" t="inlineStr"/>
       <c r="O7" s="22" t="inlineStr"/>
@@ -1931,7 +1939,11 @@
         </is>
       </c>
       <c r="K8" s="22" t="inlineStr"/>
-      <c r="L8" s="22" t="inlineStr"/>
+      <c r="L8" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M8" s="22" t="inlineStr"/>
       <c r="N8" s="22" t="inlineStr"/>
       <c r="O8" s="22" t="inlineStr"/>
@@ -1984,7 +1996,11 @@
         </is>
       </c>
       <c r="K9" s="22" t="inlineStr"/>
-      <c r="L9" s="22" t="inlineStr"/>
+      <c r="L9" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M9" s="22" t="inlineStr"/>
       <c r="N9" s="22" t="inlineStr"/>
       <c r="O9" s="22" t="inlineStr"/>
@@ -2037,7 +2053,11 @@
         </is>
       </c>
       <c r="K10" s="22" t="inlineStr"/>
-      <c r="L10" s="22" t="inlineStr"/>
+      <c r="L10" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M10" s="22" t="inlineStr"/>
       <c r="N10" s="22" t="inlineStr"/>
       <c r="O10" s="22" t="inlineStr"/>
@@ -2090,7 +2110,11 @@
         </is>
       </c>
       <c r="K11" s="22" t="inlineStr"/>
-      <c r="L11" s="22" t="inlineStr"/>
+      <c r="L11" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M11" s="22" t="inlineStr"/>
       <c r="N11" s="22" t="inlineStr"/>
       <c r="O11" s="22" t="inlineStr"/>
@@ -2143,7 +2167,11 @@
         </is>
       </c>
       <c r="K12" s="22" t="inlineStr"/>
-      <c r="L12" s="22" t="inlineStr"/>
+      <c r="L12" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M12" s="22" t="inlineStr"/>
       <c r="N12" s="22" t="inlineStr"/>
       <c r="O12" s="22" t="inlineStr"/>
@@ -2196,7 +2224,11 @@
         </is>
       </c>
       <c r="K13" s="22" t="inlineStr"/>
-      <c r="L13" s="22" t="inlineStr"/>
+      <c r="L13" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M13" s="22" t="inlineStr"/>
       <c r="N13" s="22" t="inlineStr"/>
       <c r="O13" s="22" t="inlineStr"/>
@@ -2249,7 +2281,11 @@
         </is>
       </c>
       <c r="K14" s="22" t="inlineStr"/>
-      <c r="L14" s="22" t="inlineStr"/>
+      <c r="L14" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M14" s="22" t="inlineStr"/>
       <c r="N14" s="22" t="inlineStr"/>
       <c r="O14" s="22" t="inlineStr"/>
@@ -2302,7 +2338,11 @@
         </is>
       </c>
       <c r="K15" s="22" t="inlineStr"/>
-      <c r="L15" s="22" t="inlineStr"/>
+      <c r="L15" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M15" s="22" t="inlineStr"/>
       <c r="N15" s="22" t="inlineStr"/>
       <c r="O15" s="22" t="inlineStr"/>
@@ -2355,7 +2395,11 @@
         </is>
       </c>
       <c r="K16" s="22" t="inlineStr"/>
-      <c r="L16" s="22" t="inlineStr"/>
+      <c r="L16" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M16" s="22" t="inlineStr"/>
       <c r="N16" s="22" t="inlineStr"/>
       <c r="O16" s="22" t="inlineStr"/>
@@ -2408,7 +2452,11 @@
         </is>
       </c>
       <c r="K17" s="22" t="inlineStr"/>
-      <c r="L17" s="22" t="inlineStr"/>
+      <c r="L17" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M17" s="22" t="inlineStr"/>
       <c r="N17" s="22" t="inlineStr"/>
       <c r="O17" s="22" t="inlineStr"/>
@@ -2461,7 +2509,11 @@
         </is>
       </c>
       <c r="K18" s="22" t="inlineStr"/>
-      <c r="L18" s="22" t="inlineStr"/>
+      <c r="L18" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M18" s="22" t="inlineStr"/>
       <c r="N18" s="22" t="inlineStr"/>
       <c r="O18" s="22" t="inlineStr"/>
@@ -2514,7 +2566,11 @@
         </is>
       </c>
       <c r="K19" s="22" t="inlineStr"/>
-      <c r="L19" s="22" t="inlineStr"/>
+      <c r="L19" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M19" s="22" t="inlineStr"/>
       <c r="N19" s="22" t="inlineStr"/>
       <c r="O19" s="22" t="inlineStr"/>
@@ -2567,7 +2623,11 @@
         </is>
       </c>
       <c r="K20" s="22" t="inlineStr"/>
-      <c r="L20" s="22" t="inlineStr"/>
+      <c r="L20" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M20" s="22" t="inlineStr"/>
       <c r="N20" s="22" t="inlineStr"/>
       <c r="O20" s="22" t="inlineStr"/>
@@ -2620,7 +2680,11 @@
         </is>
       </c>
       <c r="K21" s="22" t="inlineStr"/>
-      <c r="L21" s="22" t="inlineStr"/>
+      <c r="L21" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M21" s="22" t="inlineStr"/>
       <c r="N21" s="22" t="inlineStr"/>
       <c r="O21" s="22" t="inlineStr"/>
@@ -2667,7 +2731,11 @@
         </is>
       </c>
       <c r="K22" s="28" t="inlineStr"/>
-      <c r="L22" s="28" t="inlineStr"/>
+      <c r="L22" s="33" t="inlineStr">
+        <is>
+          <t>ณัช วิกรัยเจริญ</t>
+        </is>
+      </c>
       <c r="M22" s="28" t="inlineStr"/>
       <c r="N22" s="28" t="inlineStr"/>
       <c r="O22" s="28" t="inlineStr"/>

</xml_diff>